<commit_message>
before adding electricity grid
</commit_message>
<xml_diff>
--- a/case_studies/current_layout/carriers_list.xlsx
+++ b/case_studies/current_layout/carriers_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\backbone\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\current_layout_optimal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCCE35E1-1604-4AC1-99A3-CB007A028ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C504E9C-C6B4-4BA6-8253-2196AE4B5A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-360" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="carriers" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>electricity</t>
   </si>
@@ -91,6 +91,9 @@
   </si>
   <si>
     <t>CO2captured</t>
+  </si>
+  <si>
+    <t>electricity_grid</t>
   </si>
 </sst>
 </file>
@@ -417,117 +420,122 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A23"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
hydrogen_transported added to carriers_list
</commit_message>
<xml_diff>
--- a/case_studies/current_layout/carriers_list.xlsx
+++ b/case_studies/current_layout/carriers_list.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\current_layout_optimal\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\current_layout\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C504E9C-C6B4-4BA6-8253-2196AE4B5A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8C32306-735D-49BF-81EE-7E06F5EE519C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>electricity</t>
   </si>
@@ -94,6 +94,9 @@
   </si>
   <si>
     <t>electricity_grid</t>
+  </si>
+  <si>
+    <t>hydrogen_transported</t>
   </si>
 </sst>
 </file>
@@ -420,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -538,6 +541,11 @@
         <v>22</v>
       </c>
     </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>